<commit_message>
New Results and Updated Faculty List
</commit_message>
<xml_diff>
--- a/scsc_postdocs.xlsx
+++ b/scsc_postdocs.xlsx
@@ -17,13 +17,16 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -34,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -42,12 +45,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -413,56 +425,56 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J24"/>
+  <dimension ref="A1:J34"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>name</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>email</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>phone</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>title</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>unit_name</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>person_url</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>supervisor_name</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>supervisor_url</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>supervisor_phone</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -471,22 +483,22 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>Rafique Chawdhery</t>
+          <t>Bronte Sone</t>
         </is>
       </c>
       <c r="B2" t="inlineStr">
         <is>
-          <t>rafique.chawdhery@ag.tamu.edu</t>
+          <t>bronte.sone@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C2" t="inlineStr">
         <is>
-          <t>979-321-5916</t>
+          <t>979-321-5943</t>
         </is>
       </c>
       <c r="D2" t="inlineStr">
         <is>
-          <t>Postdoctoral Extension Associate</t>
+          <t>Postdoctoral Research Associate</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -496,22 +508,22 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/40370</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/40476</t>
         </is>
       </c>
       <c r="G2" t="inlineStr">
         <is>
-          <t>Jake Mowrer</t>
+          <t>Peyton Smith</t>
         </is>
       </c>
       <c r="H2" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/26177</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/29114</t>
         </is>
       </c>
       <c r="I2" t="inlineStr">
         <is>
-          <t>979-845-5366</t>
+          <t>979-845-5669</t>
         </is>
       </c>
       <c r="J2" t="inlineStr">
@@ -523,47 +535,47 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>Hatem Younes</t>
+          <t>Rafique Chawdhery</t>
         </is>
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>hatem.younes@ag.tamu.edu</t>
+          <t>rafique.chawdhery@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>830-988-6169</t>
+          <t>979-321-5916</t>
         </is>
       </c>
       <c r="D3" t="inlineStr">
         <is>
-          <t>Postdoctoral Research Associate</t>
+          <t>Postdoctoral Extension Associate</t>
         </is>
       </c>
       <c r="E3" t="inlineStr">
         <is>
-          <t>Uvalde Research and Extension Center</t>
+          <t>Soil and Crop Sciences (SCSC)</t>
         </is>
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/40259</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/40370</t>
         </is>
       </c>
       <c r="G3" t="inlineStr">
         <is>
-          <t>Xuejun Dong</t>
+          <t>Jake Mowrer</t>
         </is>
       </c>
       <c r="H3" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/24202</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/26177</t>
         </is>
       </c>
       <c r="I3" t="inlineStr">
         <is>
-          <t>830-988-6136</t>
+          <t>979-845-5366</t>
         </is>
       </c>
       <c r="J3" t="inlineStr">
@@ -575,17 +587,17 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>Md Nafiul Islam</t>
+          <t>Hatem Younes</t>
         </is>
       </c>
       <c r="B4" t="inlineStr">
         <is>
-          <t>mdnafiul.islam@ag.tamu.edu</t>
+          <t>hatem.younes@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C4" t="inlineStr">
         <is>
-          <t>979-321-5900</t>
+          <t>830-988-6169</t>
         </is>
       </c>
       <c r="D4" t="inlineStr">
@@ -595,27 +607,27 @@
       </c>
       <c r="E4" t="inlineStr">
         <is>
-          <t>Soil and Crop Sciences (SCSC)</t>
+          <t>Uvalde Research and Extension Center</t>
         </is>
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/39982</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/40259</t>
         </is>
       </c>
       <c r="G4" t="inlineStr">
         <is>
-          <t>Thanos Gentimis</t>
+          <t>Xuejun Dong</t>
         </is>
       </c>
       <c r="H4" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/39377</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/24202</t>
         </is>
       </c>
       <c r="I4" t="inlineStr">
         <is>
-          <t>979-321-5900</t>
+          <t>830-988-6136</t>
         </is>
       </c>
       <c r="J4" t="inlineStr">
@@ -627,47 +639,47 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Saven Thai</t>
+          <t>Md Nafiul Islam</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>saven.thai@ag.tamu.edu</t>
+          <t>mdnafiul.islam@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C5" t="inlineStr">
         <is>
-          <t>903-834-6191</t>
+          <t>979-321-5900</t>
         </is>
       </c>
       <c r="D5" t="inlineStr">
         <is>
-          <t>Post Doctoral Research Associate Support Staff</t>
+          <t>Postdoctoral Research Associate</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
         <is>
-          <t>Overton Research and Extension Center</t>
+          <t>Soil and Crop Sciences (SCSC)</t>
         </is>
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/39136</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/39982</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>Anil Somenahally</t>
+          <t>Thanos Gentimis</t>
         </is>
       </c>
       <c r="H5" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/18157</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/39377</t>
         </is>
       </c>
       <c r="I5" t="inlineStr">
         <is>
-          <t>903-834-6191</t>
+          <t>979-321-5900</t>
         </is>
       </c>
       <c r="J5" t="inlineStr">
@@ -679,22 +691,22 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>Tajamul Hussain</t>
+          <t>Nataleigh Perez</t>
         </is>
       </c>
       <c r="B6" t="inlineStr">
         <is>
-          <t>tajamul.hussain@ag.tamu.edu</t>
+          <t>nataleigh.perez@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>979-321-5900</t>
+          <t>979-321-5920</t>
         </is>
       </c>
       <c r="D6" t="inlineStr">
         <is>
-          <t>Postdoctoral Extension Associate</t>
+          <t>Postdoctoral Research Associate</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -704,22 +716,22 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/38854</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/39318</t>
         </is>
       </c>
       <c r="G6" t="inlineStr">
         <is>
-          <t>Reagan Noland</t>
+          <t>Felipe Aburto</t>
         </is>
       </c>
       <c r="H6" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/14035</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/33506</t>
         </is>
       </c>
       <c r="I6" t="inlineStr">
         <is>
-          <t>325-653-4576</t>
+          <t>979-845-3603</t>
         </is>
       </c>
       <c r="J6" t="inlineStr">
@@ -731,47 +743,47 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>DrDeepak Loura Facebook Instagram LinkedIn</t>
+          <t>Saven Thai</t>
         </is>
       </c>
       <c r="B7" t="inlineStr">
         <is>
-          <t>deepak.loura@ag.tamu.edu</t>
+          <t>saven.thai@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C7" t="inlineStr">
         <is>
-          <t>979-344-9177</t>
+          <t>903-834-6191</t>
         </is>
       </c>
       <c r="D7" t="inlineStr">
         <is>
-          <t>Postdoctoral Research Associate</t>
+          <t>Post Doctoral Research Associate Support Staff</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>Soil and Crop Sciences (SCSC)</t>
+          <t>Overton Research and Extension Center</t>
         </is>
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/38227</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/39136</t>
         </is>
       </c>
       <c r="G7" t="inlineStr">
         <is>
-          <t>Muthu Bagavathiannan</t>
+          <t>Anil Somenahally</t>
         </is>
       </c>
       <c r="H7" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/24878</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/18157</t>
         </is>
       </c>
       <c r="I7" t="inlineStr">
         <is>
-          <t>979-845-3041</t>
+          <t>903-834-6191</t>
         </is>
       </c>
       <c r="J7" t="inlineStr">
@@ -783,47 +795,47 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>Daniel Cudjoe</t>
+          <t>Tajamul Hussain</t>
         </is>
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>daniel.cudjoe@ag.tamu.edu</t>
+          <t>tajamul.hussain@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C8" t="inlineStr">
         <is>
-          <t>806-746-6101</t>
+          <t>979-321-5900</t>
         </is>
       </c>
       <c r="D8" t="inlineStr">
         <is>
-          <t>Post Doctoral Research Associate</t>
+          <t>Postdoctoral Extension Associate</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>Lubbock Research and Extension Center</t>
+          <t>Soil and Crop Sciences (SCSC)</t>
         </is>
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/38160</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/38854</t>
         </is>
       </c>
       <c r="G8" t="inlineStr">
         <is>
-          <t>Wenxuan Guo</t>
+          <t>Reagan Noland</t>
         </is>
       </c>
       <c r="H8" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/30742</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/14035</t>
         </is>
       </c>
       <c r="I8" t="inlineStr">
         <is>
-          <t>806-746-6101</t>
+          <t>325-653-4576</t>
         </is>
       </c>
       <c r="J8" t="inlineStr">
@@ -835,17 +847,17 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>Rahmatullah Hashimi LinkedIn</t>
+          <t>Shweta Panjwani</t>
         </is>
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>rahmatullah.hashimi@ag.tamu.edu</t>
+          <t>shweta.panjwani@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C9" t="inlineStr">
         <is>
-          <t>915-701-3265</t>
+          <t>254-774-6026</t>
         </is>
       </c>
       <c r="D9" t="inlineStr">
@@ -855,27 +867,27 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>El Paso Research and Extension Center</t>
+          <t>Temple Research and Extension Center</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/37969</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/38612</t>
         </is>
       </c>
       <c r="G9" t="inlineStr">
         <is>
-          <t>Girisha Ganjegunte</t>
+          <t>Gurjinder Baath</t>
         </is>
       </c>
       <c r="H9" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/6286</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/33791</t>
         </is>
       </c>
       <c r="I9" t="inlineStr">
         <is>
-          <t>915-859-9111</t>
+          <t>254-774-6017</t>
         </is>
       </c>
       <c r="J9" t="inlineStr">
@@ -887,17 +899,17 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>Uzair Ahmad</t>
+          <t>Jaydeo Dharpure</t>
         </is>
       </c>
       <c r="B10" t="inlineStr">
         <is>
-          <t>uzair.ahmad@ag.tamu.edu</t>
+          <t>jaydeo.dharpure@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C10" t="inlineStr">
         <is>
-          <t>830-988-6140</t>
+          <t>254-774-6015</t>
         </is>
       </c>
       <c r="D10" t="inlineStr">
@@ -907,27 +919,27 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>Uvalde Research and Extension Center</t>
+          <t>Temple Research and Extension Center</t>
         </is>
       </c>
       <c r="F10" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/37916</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/38606</t>
         </is>
       </c>
       <c r="G10" t="inlineStr">
         <is>
-          <t>Xuejun Dong</t>
+          <t>Gurjinder Baath</t>
         </is>
       </c>
       <c r="H10" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/24202</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/33791</t>
         </is>
       </c>
       <c r="I10" t="inlineStr">
         <is>
-          <t>830-988-6136</t>
+          <t>254-774-6017</t>
         </is>
       </c>
       <c r="J10" t="inlineStr">
@@ -939,47 +951,47 @@
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>Arjun Kafle</t>
+          <t>DrDeepak Loura Facebook Instagram LinkedIn</t>
         </is>
       </c>
       <c r="B11" t="inlineStr">
         <is>
-          <t>arjun.kafle@ag.tamu.edu</t>
+          <t>deepak.loura@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C11" t="inlineStr">
         <is>
-          <t>806-746-6101</t>
+          <t>979-344-9177</t>
         </is>
       </c>
       <c r="D11" t="inlineStr">
         <is>
-          <t>Postdoctoral Research Associate Soil Fertility</t>
+          <t>Postdoctoral Research Associate</t>
         </is>
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>Lubbock Research and Extension Center</t>
+          <t>Soil and Crop Sciences (SCSC)</t>
         </is>
       </c>
       <c r="F11" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/37857</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/38227</t>
         </is>
       </c>
       <c r="G11" t="inlineStr">
         <is>
-          <t>Katie Lewis</t>
+          <t>Muthu Bagavathiannan</t>
         </is>
       </c>
       <c r="H11" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/16614</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/24878</t>
         </is>
       </c>
       <c r="I11" t="inlineStr">
         <is>
-          <t>806-746-6101</t>
+          <t>979-845-3041</t>
         </is>
       </c>
       <c r="J11" t="inlineStr">
@@ -991,17 +1003,17 @@
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
-          <t>Fidel Gonzalez Torralva</t>
+          <t>Daniel Cudjoe</t>
         </is>
       </c>
       <c r="B12" t="inlineStr">
         <is>
-          <t>fid.gonzaleztorralva@ag.tamu.edu</t>
+          <t>daniel.cudjoe@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C12" t="inlineStr">
         <is>
-          <t>409-752-2741</t>
+          <t>806-746-6101</t>
         </is>
       </c>
       <c r="D12" t="inlineStr">
@@ -1011,27 +1023,27 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>Beaumont Research Center</t>
+          <t>Lubbock Research and Extension Center</t>
         </is>
       </c>
       <c r="F12" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/36839</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/38160</t>
         </is>
       </c>
       <c r="G12" t="inlineStr">
         <is>
-          <t>Mithila Jugulam</t>
+          <t>Wenxuan Guo</t>
         </is>
       </c>
       <c r="H12" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/38032</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/30742</t>
         </is>
       </c>
       <c r="I12" t="inlineStr">
         <is>
-          <t>409-752-2741</t>
+          <t>806-746-6101</t>
         </is>
       </c>
       <c r="J12" t="inlineStr">
@@ -1043,47 +1055,47 @@
     <row r="13">
       <c r="A13" t="inlineStr">
         <is>
-          <t>Pablo Guarnido Lopez</t>
+          <t>Mohammed Omer</t>
         </is>
       </c>
       <c r="B13" t="inlineStr">
         <is>
-          <t>pablo.guarnidolopez@ag.tamu.edu</t>
+          <t>mohammed.omer@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C13" t="inlineStr">
         <is>
-          <t>361-698-7400</t>
+          <t>972-231-5362</t>
         </is>
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>Post Doctoral Research Associate</t>
+          <t>Postdoctoral Research Associate</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>Corpus Christi Research and Extension Center</t>
+          <t>Dallas Research and Extension Center</t>
         </is>
       </c>
       <c r="F13" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/36555</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/38084</t>
         </is>
       </c>
       <c r="G13" t="inlineStr">
         <is>
-          <t>Jamie Foster</t>
+          <t>Pablo Boeri</t>
         </is>
       </c>
       <c r="H13" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/5963</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/36757</t>
         </is>
       </c>
       <c r="I13" t="inlineStr">
         <is>
-          <t>361-360-4536</t>
+          <t>972-231-5362</t>
         </is>
       </c>
       <c r="J13" t="inlineStr">
@@ -1095,17 +1107,17 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Gurjeet Singh</t>
+          <t>Rahmatullah Hashimi LinkedIn</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>gurjeet.singh@ag.tamu.edu</t>
+          <t>rahmatullah.hashimi@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C14" t="inlineStr">
         <is>
-          <t>409-752-2741</t>
+          <t>915-701-3265</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
@@ -1115,27 +1127,27 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>Beaumont Research Center</t>
+          <t>El Paso Research and Extension Center</t>
         </is>
       </c>
       <c r="F14" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/35188</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/37969</t>
         </is>
       </c>
       <c r="G14" t="inlineStr">
         <is>
-          <t>Shyamal Talukder</t>
+          <t>Girisha Ganjegunte</t>
         </is>
       </c>
       <c r="H14" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/33125</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/6286</t>
         </is>
       </c>
       <c r="I14" t="inlineStr">
         <is>
-          <t>409-245-8623</t>
+          <t>915-859-9111</t>
         </is>
       </c>
       <c r="J14" t="inlineStr">
@@ -1147,17 +1159,17 @@
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>Andrea Leiva Soto</t>
+          <t>Uzair Ahmad</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>andrea.leivasoto@ag.tamu.edu</t>
+          <t>uzair.ahmad@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C15" t="inlineStr">
         <is>
-          <t>806-354-5810</t>
+          <t>830-988-6140</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
@@ -1167,27 +1179,27 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>High Plains Research and Extension Center</t>
+          <t>Uvalde Research and Extension Center</t>
         </is>
       </c>
       <c r="F15" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/34459</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/37916</t>
         </is>
       </c>
       <c r="G15" t="inlineStr">
         <is>
-          <t>Qingwu Xue</t>
+          <t>Xuejun Dong</t>
         </is>
       </c>
       <c r="H15" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/21433</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/24202</t>
         </is>
       </c>
       <c r="I15" t="inlineStr">
         <is>
-          <t>806-354-5803</t>
+          <t>830-988-6136</t>
         </is>
       </c>
       <c r="J15" t="inlineStr">
@@ -1199,47 +1211,47 @@
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>Lei Zhao</t>
+          <t>Arjun Kafle</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>lei.zhao@ag.tamu.edu</t>
+          <t>arjun.kafle@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>361-698-7400</t>
+          <t>806-746-6101</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>Postdoctoral Research Associate</t>
+          <t>Postdoctoral Research Associate Soil Fertility</t>
         </is>
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>Corpus Christi Research and Extension Center</t>
+          <t>Lubbock Research and Extension Center</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/34281</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/37857</t>
         </is>
       </c>
       <c r="G16" t="inlineStr">
         <is>
-          <t>Mahendra Bhandari</t>
+          <t>Katie Lewis</t>
         </is>
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/28204</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/16614</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
         <is>
-          <t>361-698-7400</t>
+          <t>806-746-6101</t>
         </is>
       </c>
       <c r="J16" t="inlineStr">
@@ -1251,17 +1263,17 @@
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>Basu Kafle</t>
+          <t>Fidel Gonzalez Torralva</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>basu.kafle@ag.tamu.edu</t>
+          <t>fid.gonzaleztorralva@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>254-968-4144</t>
+          <t>409-752-2741</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
@@ -1271,27 +1283,27 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>Stephenville Research and Extension Center</t>
+          <t>Beaumont Research Center</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/33156</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/36839</t>
         </is>
       </c>
       <c r="G17" t="inlineStr">
         <is>
-          <t>John Cason</t>
+          <t>Mithila Jugulam</t>
         </is>
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/2917</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/38032</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
         <is>
-          <t>254-968-4144</t>
+          <t>409-752-2741</t>
         </is>
       </c>
       <c r="J17" t="inlineStr">
@@ -1303,22 +1315,22 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>William Wheeler</t>
+          <t>Jialin Hu</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>william.wheeler@ag.tamu.edu</t>
+          <t>jialin.hu@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>979-845-3041</t>
+          <t>979-321-5918</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>Postdoctoral Research Associate</t>
+          <t>Post Doctoral Research Associate</t>
         </is>
       </c>
       <c r="E18" t="inlineStr">
@@ -1328,17 +1340,17 @@
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/32947</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/36640</t>
         </is>
       </c>
       <c r="G18" t="inlineStr">
         <is>
-          <t>Nithya Rajan</t>
+          <t>Terry Gentry</t>
         </is>
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/15613</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/6569</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -1355,47 +1367,47 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>Sudip Biswas</t>
+          <t>Pablo Guarnido Lopez</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>sudip.biswas@ag.tamu.edu</t>
+          <t>pablo.guarnidolopez@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>979-845-3041</t>
+          <t>361-698-7400</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>Post Doctoral Research</t>
+          <t>Post Doctoral Research Associate</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>Soil and Crop Sciences (SCSC)</t>
+          <t>Corpus Christi Research and Extension Center</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/32319</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/36555</t>
         </is>
       </c>
       <c r="G19" t="inlineStr">
         <is>
-          <t>Endang Septiningsih</t>
+          <t>Jamie Foster</t>
         </is>
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/26253</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/5963</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>979-845-3041</t>
+          <t>361-360-4536</t>
         </is>
       </c>
       <c r="J19" t="inlineStr">
@@ -1407,17 +1419,17 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>Suman Lamichhane</t>
+          <t>Md Zakaria Hossain Prodhan</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>suman.lamichhane@ag.tamu.edu</t>
+          <t>mdzakaria.prodhan@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>409-245-8625</t>
+          <t>409-752-2741</t>
         </is>
       </c>
       <c r="D20" t="inlineStr">
@@ -1432,22 +1444,22 @@
       </c>
       <c r="F20" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/31317</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/36444</t>
         </is>
       </c>
       <c r="G20" t="inlineStr">
         <is>
-          <t>Fugen Dou</t>
+          <t>Stanley Samonte</t>
         </is>
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/4814</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/16880</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>409-245-8611</t>
+          <t>409-245-8624</t>
         </is>
       </c>
       <c r="J20" t="inlineStr">
@@ -1459,47 +1471,47 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>Rajan Shrestha</t>
+          <t>Wen-Hui Li</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>rajan.shrestha@ag.tamu.edu</t>
+          <t>wen-hui.li@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>806-354-5814</t>
+          <t>979-321-5904</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>Postdoctoral Research Associate Support Staff</t>
+          <t>Postdoctoral Research Associate</t>
         </is>
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>High Plains Research and Extension Center</t>
+          <t>Soil and Crop Sciences (SCSC)</t>
         </is>
       </c>
       <c r="F21" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/29366</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/36391</t>
         </is>
       </c>
       <c r="G21" t="inlineStr">
         <is>
-          <t>Qingwu Xue</t>
+          <t>Julie Howe</t>
         </is>
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/21433</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/27971</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>806-354-5803</t>
+          <t>979-845-3041</t>
         </is>
       </c>
       <c r="J21" t="inlineStr">
@@ -1511,17 +1523,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>Jhaman Suthar</t>
+          <t>Gurjeet Singh</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
-          <t>jhaman.suthar@ag.tamu.edu</t>
+          <t>gurjeet.singh@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>915-859-9111</t>
+          <t>409-752-2741</t>
         </is>
       </c>
       <c r="D22" t="inlineStr">
@@ -1531,27 +1543,27 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>El Paso Research and Extension Center</t>
+          <t>Beaumont Research Center</t>
         </is>
       </c>
       <c r="F22" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/28466</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/35188</t>
         </is>
       </c>
       <c r="G22" t="inlineStr">
         <is>
-          <t>Girisha Ganjegunte</t>
+          <t>Shyamal Talukder</t>
         </is>
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/6286</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/33125</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>915-859-9111</t>
+          <t>409-245-8623</t>
         </is>
       </c>
       <c r="J22" t="inlineStr">
@@ -1563,47 +1575,47 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>Ahmed Attia</t>
+          <t>Andrea Leiva Soto</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
-          <t>ahmed.attia@ag.tamu.edu</t>
+          <t>andrea.leivasoto@ag.tamu.edu</t>
         </is>
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>903-834-6191</t>
+          <t>806-354-5810</t>
         </is>
       </c>
       <c r="D23" t="inlineStr">
         <is>
-          <t>Postdoctoral Research Associate Support Staff</t>
+          <t>Postdoctoral Research Associate</t>
         </is>
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>Overton Research and Extension Center</t>
+          <t>High Plains Research and Extension Center</t>
         </is>
       </c>
       <c r="F23" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/22652</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/34459</t>
         </is>
       </c>
       <c r="G23" t="inlineStr">
         <is>
-          <t>Prem Oli</t>
+          <t>Qingwu Xue</t>
         </is>
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>https://agrilifepeople.tamu.edu/people/view/27002</t>
+          <t>https://agrilifepeople.tamu.edu/people/view/21433</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>903-834-6191</t>
+          <t>806-354-5803</t>
         </is>
       </c>
       <c r="J23" t="inlineStr">
@@ -1615,50 +1627,570 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
+          <t>Lei Zhao</t>
+        </is>
+      </c>
+      <c r="B24" t="inlineStr">
+        <is>
+          <t>lei.zhao@ag.tamu.edu</t>
+        </is>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>361-698-7400</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>Postdoctoral Research Associate</t>
+        </is>
+      </c>
+      <c r="E24" t="inlineStr">
+        <is>
+          <t>Corpus Christi Research and Extension Center</t>
+        </is>
+      </c>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/34281</t>
+        </is>
+      </c>
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>Mahendra Bhandari</t>
+        </is>
+      </c>
+      <c r="H24" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/28204</t>
+        </is>
+      </c>
+      <c r="I24" t="inlineStr">
+        <is>
+          <t>361-698-7400</t>
+        </is>
+      </c>
+      <c r="J24" t="inlineStr">
+        <is>
+          <t>OLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" t="inlineStr">
+        <is>
+          <t>Basu Kafle</t>
+        </is>
+      </c>
+      <c r="B25" t="inlineStr">
+        <is>
+          <t>basu.kafle@ag.tamu.edu</t>
+        </is>
+      </c>
+      <c r="C25" t="inlineStr">
+        <is>
+          <t>254-968-4144</t>
+        </is>
+      </c>
+      <c r="D25" t="inlineStr">
+        <is>
+          <t>Post Doctoral Research Associate</t>
+        </is>
+      </c>
+      <c r="E25" t="inlineStr">
+        <is>
+          <t>Stephenville Research and Extension Center</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/33156</t>
+        </is>
+      </c>
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>John Cason</t>
+        </is>
+      </c>
+      <c r="H25" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/2917</t>
+        </is>
+      </c>
+      <c r="I25" t="inlineStr">
+        <is>
+          <t>254-968-4144</t>
+        </is>
+      </c>
+      <c r="J25" t="inlineStr">
+        <is>
+          <t>OLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>William Wheeler</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>william.wheeler@ag.tamu.edu</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>979-845-3041</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>Postdoctoral Research Associate</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>Soil and Crop Sciences (SCSC)</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/32947</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>Nithya Rajan</t>
+        </is>
+      </c>
+      <c r="H26" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/15613</t>
+        </is>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>979-845-3041</t>
+        </is>
+      </c>
+      <c r="J26" t="inlineStr">
+        <is>
+          <t>OLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>Sudip Biswas</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>sudip.biswas@ag.tamu.edu</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>979-845-3041</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>Post Doctoral Research</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>Soil and Crop Sciences (SCSC)</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/32319</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>Endang Septiningsih</t>
+        </is>
+      </c>
+      <c r="H27" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/26253</t>
+        </is>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>979-845-3041</t>
+        </is>
+      </c>
+      <c r="J27" t="inlineStr">
+        <is>
+          <t>OLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>Bala Sapkota</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>bala.sapkota@ag.tamu.edu</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>254-774-6037</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>Post Doctoral Research Associate</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>Temple Research and Extension Center</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/31943</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>Gurjinder Baath</t>
+        </is>
+      </c>
+      <c r="H28" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/33791</t>
+        </is>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>254-774-6017</t>
+        </is>
+      </c>
+      <c r="J28" t="inlineStr">
+        <is>
+          <t>OLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>Ellen Melson</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>ellen.melson@ag.tamu.edu</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>979-845-3041</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>Postdoctoral Research Associate</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>Soil and Crop Sciences (SCSC)</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/31759</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>Russell Sutton</t>
+        </is>
+      </c>
+      <c r="H29" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/18817</t>
+        </is>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>979-845-3041</t>
+        </is>
+      </c>
+      <c r="J29" t="inlineStr">
+        <is>
+          <t>OLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>Suman Lamichhane</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>suman.lamichhane@ag.tamu.edu</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>409-245-8625</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>Postdoctoral Research Associate</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>Beaumont Research Center</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/31317</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>Fugen Dou</t>
+        </is>
+      </c>
+      <c r="H30" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/4814</t>
+        </is>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>409-245-8611</t>
+        </is>
+      </c>
+      <c r="J30" t="inlineStr">
+        <is>
+          <t>OLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>Rajan Shrestha</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>rajan.shrestha@ag.tamu.edu</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>806-354-5814</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>Postdoctoral Research Associate Support Staff</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>High Plains Research and Extension Center</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/29366</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>Qingwu Xue</t>
+        </is>
+      </c>
+      <c r="H31" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/21433</t>
+        </is>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>806-354-5803</t>
+        </is>
+      </c>
+      <c r="J31" t="inlineStr">
+        <is>
+          <t>OLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>Jhaman Suthar</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>jhaman.suthar@ag.tamu.edu</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>915-859-9111</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>Postdoctoral Research Associate</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>El Paso Research and Extension Center</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/28466</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>Girisha Ganjegunte</t>
+        </is>
+      </c>
+      <c r="H32" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/6286</t>
+        </is>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>915-859-9111</t>
+        </is>
+      </c>
+      <c r="J32" t="inlineStr">
+        <is>
+          <t>OLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>Ahmed Attia</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>ahmed.attia@ag.tamu.edu</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>903-834-6191</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>Postdoctoral Research Associate Support Staff</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>Overton Research and Extension Center</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/22652</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>Prem Oli</t>
+        </is>
+      </c>
+      <c r="H33" t="inlineStr">
+        <is>
+          <t>https://agrilifepeople.tamu.edu/people/view/27002</t>
+        </is>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>903-834-6191</t>
+        </is>
+      </c>
+      <c r="J33" t="inlineStr">
+        <is>
+          <t>OLD</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
           <t>Jennifer Chagoya</t>
         </is>
       </c>
-      <c r="B24" t="inlineStr">
+      <c r="B34" t="inlineStr">
         <is>
           <t>jennifer.chagoya@ag.tamu.edu</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr">
+      <c r="C34" t="inlineStr">
         <is>
           <t>806-746-6101</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr">
+      <c r="D34" t="inlineStr">
         <is>
           <t>Administrative Postdoctoral Associate</t>
         </is>
       </c>
-      <c r="E24" t="inlineStr">
+      <c r="E34" t="inlineStr">
         <is>
           <t>Lubbock Research and Extension Center</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr">
+      <c r="F34" t="inlineStr">
         <is>
           <t>https://agrilifepeople.tamu.edu/people/view/3053</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr">
+      <c r="G34" t="inlineStr">
         <is>
           <t>Carol Kelly</t>
         </is>
       </c>
-      <c r="H24" t="inlineStr">
+      <c r="H34" t="inlineStr">
         <is>
           <t>https://agrilifepeople.tamu.edu/people/view/9843</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr">
+      <c r="I34" t="inlineStr">
         <is>
           <t>806-746-6101</t>
         </is>
       </c>
-      <c r="J24" t="inlineStr">
+      <c r="J34" t="inlineStr">
         <is>
           <t>OLD</t>
         </is>

</xml_diff>